<commit_message>
Pasar justificacion y detalle de gastos a US$ 27,000 hasta fin de 2026
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DoHx9ZQNZXcgog7oJGoyRL
</commit_message>
<xml_diff>
--- a/detalle-gastos-desercion-vehicular.xlsx
+++ b/detalle-gastos-desercion-vehicular.xlsx
@@ -20,12 +20,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
   <si>
     <t xml:space="preserve">Ampliacion de OC - ESTRATEK S.A.S. SUCURSAL DEL PERU - Iniciativa de Desercion Vehicular</t>
   </si>
   <si>
-    <t xml:space="preserve">Sustento del monto de la ampliacion (S/ 27,000 sin IGV) para 75 dias (2.5 meses).</t>
+    <t xml:space="preserve">Detalle de gastos en dolares (US$). Monto tope: US$ 27,000 + IGV, hasta el 31 de diciembre de 2026.</t>
   </si>
   <si>
     <t xml:space="preserve">Leyenda:</t>
@@ -37,34 +37,25 @@
     <t xml:space="preserve">Celda calculada</t>
   </si>
   <si>
-    <t xml:space="preserve">SUPUESTOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Monto de la ampliacion de OC (S/, sin IGV)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Registros objetivo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Costo plataforma por registro (US$, incluye conversaciones del chatbot)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tipo de cambio (S/ por US$) - SUPUESTO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bono diario equipo de volanteo (S/)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dias que trabaja el equipo por mes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Meses de ejecucion</t>
+    <t xml:space="preserve">DATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Monto tope de la ampliacion (US$, sin IGV)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Registros</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Costo por registro (US$, incluye conversaciones del chatbot)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% del saldo para marketing digital (el resto va a volanteo)</t>
   </si>
   <si>
     <t xml:space="preserve">IGV</t>
   </si>
   <si>
-    <t xml:space="preserve">DETALLE DE GASTOS</t>
+    <t xml:space="preserve">DETALLE DE GASTOS (US$)</t>
   </si>
   <si>
     <t xml:space="preserve">Componente</t>
@@ -73,7 +64,7 @@
     <t xml:space="preserve">Calculo</t>
   </si>
   <si>
-    <t xml:space="preserve">Monto (S/)</t>
+    <t xml:space="preserve">Monto (US$)</t>
   </si>
   <si>
     <t xml:space="preserve">% del total</t>
@@ -82,19 +73,19 @@
     <t xml:space="preserve">1. Plataforma de registros y chatbot</t>
   </si>
   <si>
-    <t xml:space="preserve">Registros x US$ 0.80 x tipo de cambio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2. Volanteo en campo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bono diario x dias/mes x meses</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. Marketing digital</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Saldo del monto para campanas de captacion</t>
+    <t xml:space="preserve">Registros x costo por registro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Marketing digital</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saldo x % para marketing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Volanteo en campo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saldo restante</t>
   </si>
   <si>
     <t xml:space="preserve">VALOR NETO (sin IGV)</t>
@@ -115,56 +106,19 @@
     <t xml:space="preserve">Valor neto + IGV</t>
   </si>
   <si>
-    <t xml:space="preserve">CONTROLES</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Plataforma en US$</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Marketing digital por registro (S/)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Costo total por registro (S/, sin IGV)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Maximo de registros que cubre el monto (si marketing = 0)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Validacion</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Notas:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">- ESTRATEK S.A.S. SUCURSAL DEL PERU es el proveedor de la OC: ejecuta la iniciativa de forma integral y coordina a sus aliados especializados. Se emite una sola factura a Calidda.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">- Plataforma: US$ 0.80 por registro, que incluye las conversaciones del chatbot con el conductor. Se paga solo por registro obtenido.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">- Volanteo: bono de equipo de S/ 150/dia (rango negociado S/ 120-160) durante 2.5 meses. No depende del numero de registros.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">- Marketing digital: es el saldo del monto de la ampliacion. Si cambian los registros o el tipo de cambio, se recalcula solo.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">- El monto es un tope: si no se llega a los registros objetivo, no se ejecuta todo el gasto.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="9">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="&quot;S/ &quot;#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="&quot;US$ &quot;#,##0.00"/>
     <numFmt numFmtId="166" formatCode="#,##0"/>
-    <numFmt numFmtId="167" formatCode="&quot;US$ &quot;#,##0.00"/>
-    <numFmt numFmtId="168" formatCode="0.00"/>
-    <numFmt numFmtId="169" formatCode="0"/>
-    <numFmt numFmtId="170" formatCode="0.0"/>
-    <numFmt numFmtId="171" formatCode="0%"/>
-    <numFmt numFmtId="172" formatCode="0.0%"/>
+    <numFmt numFmtId="167" formatCode="0%"/>
+    <numFmt numFmtId="168" formatCode="0.0%"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -287,7 +241,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="15">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -320,22 +274,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="171" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -348,7 +286,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -360,24 +298,8 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="168" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -632,11 +554,11 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D36"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="60"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
   </cols>
@@ -680,14 +602,14 @@
         <v>7</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>5000</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="7" t="n">
+      <c r="B8" s="5" t="n">
         <v>0.8</v>
       </c>
     </row>
@@ -695,254 +617,137 @@
       <c r="A9" s="0" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="8" t="n">
-        <v>3.4</v>
+      <c r="B9" s="7" t="n">
+        <v>0.5</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="5" t="n">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+      <c r="B10" s="7" t="n">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="9" t="n">
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C14" s="10" t="n">
+        <f aca="false">B7*B8</f>
+        <v>8000</v>
+      </c>
+      <c r="D14" s="11" t="n">
+        <f aca="false">C14/$C$17</f>
+        <v>0.296296296296296</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="C15" s="10" t="n">
+        <f aca="false">(B6-C14)*B9</f>
+        <v>9500</v>
+      </c>
+      <c r="D15" s="11" t="n">
+        <f aca="false">C15/$C$17</f>
+        <v>0.351851851851852</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="C16" s="10" t="n">
+        <f aca="false">B6-C14-C15</f>
+        <v>9500</v>
+      </c>
+      <c r="D16" s="11" t="n">
+        <f aca="false">C16/$C$17</f>
+        <v>0.351851851851852</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="C17" s="13" t="n">
+        <f aca="false">C14+C15+C16</f>
+        <v>27000</v>
+      </c>
+      <c r="D17" s="14" t="n">
+        <f aca="false">C17/$C$17</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="C18" s="13" t="n">
+        <f aca="false">C17*B10</f>
+        <v>4860</v>
+      </c>
+      <c r="D18" s="12"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="12" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="B12" s="10" t="n">
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="B13" s="11" t="n">
-        <v>0.18</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="B16" s="12" t="s">
-        <v>16</v>
-      </c>
-      <c r="C16" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="D16" s="12" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="B17" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="C17" s="14" t="n">
-        <f aca="false">B7*B8*B9</f>
-        <v>13600</v>
-      </c>
-      <c r="D17" s="15" t="n">
-        <f aca="false">C17/$C$20</f>
-        <v>0.503703703703704</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="B18" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="C18" s="14" t="n">
-        <f aca="false">B10*B11*B12</f>
-        <v>9750</v>
-      </c>
-      <c r="D18" s="15" t="n">
-        <f aca="false">C18/$C$20</f>
-        <v>0.361111111111111</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="B19" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="C19" s="14" t="n">
-        <f aca="false">B6-C17-C18</f>
-        <v>3650</v>
-      </c>
-      <c r="D19" s="15" t="n">
-        <f aca="false">C19/$C$20</f>
-        <v>0.135185185185185</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="16" t="s">
-        <v>25</v>
-      </c>
-      <c r="B20" s="16" t="s">
-        <v>26</v>
-      </c>
-      <c r="C20" s="17" t="n">
-        <f aca="false">C17+C18+C19</f>
-        <v>27000</v>
-      </c>
-      <c r="D20" s="18" t="n">
-        <f aca="false">C20/$C$20</f>
-        <v>1</v>
-      </c>
+      <c r="B19" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="C19" s="13" t="n">
+        <f aca="false">C17+C18</f>
+        <v>31860</v>
+      </c>
+      <c r="D19" s="12"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="B21" s="16" t="s">
+      <c r="A21" s="0" t="s">
         <v>28</v>
       </c>
-      <c r="C21" s="17" t="n">
-        <f aca="false">C20*B13</f>
-        <v>4860</v>
-      </c>
-      <c r="D21" s="16"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="16" t="s">
-        <v>29</v>
-      </c>
-      <c r="B22" s="16" t="s">
-        <v>30</v>
-      </c>
-      <c r="C22" s="17" t="n">
-        <f aca="false">C20+C21</f>
-        <v>31860</v>
-      </c>
-      <c r="D22" s="16"/>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="4" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="0" t="s">
-        <v>32</v>
-      </c>
-      <c r="C25" s="19" t="n">
-        <f aca="false">B7*B8</f>
-        <v>4000</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="0" t="s">
-        <v>33</v>
-      </c>
-      <c r="C26" s="20" t="n">
-        <f aca="false">C19/B7</f>
-        <v>0.73</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="C27" s="20" t="n">
-        <f aca="false">C20/B7</f>
-        <v>5.4</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="0" t="s">
-        <v>35</v>
-      </c>
-      <c r="C28" s="21" t="n">
-        <f aca="false">ROUNDDOWN((B6-C18)/(B8*B9),0)</f>
-        <v>6341</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="0" t="s">
-        <v>36</v>
-      </c>
-      <c r="C29" s="3" t="str">
-        <f aca="false">IF(C19&lt;0,"El monto no alcanza: baja los registros","OK - el detalle suma el monto de la ampliacion")</f>
-        <v>OK - el detalle suma el monto de la ampliacion</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="4" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="B32" s="22"/>
-      <c r="C32" s="22"/>
-      <c r="D32" s="22"/>
-    </row>
-    <row r="33" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="B33" s="22"/>
-      <c r="C33" s="22"/>
-      <c r="D33" s="22"/>
-    </row>
-    <row r="34" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="B34" s="22"/>
-      <c r="C34" s="22"/>
-      <c r="D34" s="22"/>
-    </row>
-    <row r="35" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="22" t="s">
-        <v>41</v>
-      </c>
-      <c r="B35" s="22"/>
-      <c r="C35" s="22"/>
-      <c r="D35" s="22"/>
-    </row>
-    <row r="36" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="22" t="s">
-        <v>42</v>
-      </c>
-      <c r="B36" s="22"/>
-      <c r="C36" s="22"/>
-      <c r="D36" s="22"/>
+      <c r="C21" s="3" t="str">
+        <f aca="false">IF(C16&lt;0,"El monto no alcanza","OK - el detalle suma el monto tope")</f>
+        <v>OK - el detalle suma el monto tope</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A32:D32"/>
-    <mergeCell ref="A33:D33"/>
-    <mergeCell ref="A34:D34"/>
-    <mergeCell ref="A35:D35"/>
-    <mergeCell ref="A36:D36"/>
-  </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
Ajustar montos para que el total incluido IGV sea US$ 27,000
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DoHx9ZQNZXcgog7oJGoyRL
</commit_message>
<xml_diff>
--- a/detalle-gastos-desercion-vehicular.xlsx
+++ b/detalle-gastos-desercion-vehicular.xlsx
@@ -20,12 +20,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t xml:space="preserve">Ampliacion de OC - ESTRATEK S.A.S. SUCURSAL DEL PERU - Iniciativa de Desercion Vehicular</t>
   </si>
   <si>
-    <t xml:space="preserve">Detalle de gastos en dolares (US$). Monto tope: US$ 27,000 + IGV, hasta el 31 de diciembre de 2026.</t>
+    <t xml:space="preserve">Detalle de gastos en dolares (US$). Monto tope: US$ 27,000 incluido IGV, hasta el 31 de diciembre de 2026.</t>
   </si>
   <si>
     <t xml:space="preserve">Leyenda:</t>
@@ -40,7 +40,7 @@
     <t xml:space="preserve">DATOS</t>
   </si>
   <si>
-    <t xml:space="preserve">Monto tope de la ampliacion (US$, sin IGV)</t>
+    <t xml:space="preserve">Monto tope de la ampliacion (US$, incluido IGV)</t>
   </si>
   <si>
     <t xml:space="preserve">Registros</t>
@@ -53,6 +53,9 @@
   </si>
   <si>
     <t xml:space="preserve">IGV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valor neto disponible (US$, sin IGV)</t>
   </si>
   <si>
     <t xml:space="preserve">DETALLE DE GASTOS (US$)</t>
@@ -274,15 +277,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -629,83 +632,92 @@
         <v>0.18</v>
       </c>
     </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11" s="8" t="n">
+        <f aca="false">B6/(1+B10)</f>
+        <v>22881.3559322034</v>
+      </c>
+    </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="B13" s="8" t="s">
+      <c r="A13" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="C13" s="8" t="s">
+      <c r="B13" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="D13" s="8" t="s">
+      <c r="C13" s="9" t="s">
         <v>15</v>
       </c>
+      <c r="D13" s="9" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="B14" s="9" t="s">
+      <c r="A14" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="C14" s="10" t="n">
+      <c r="B14" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" s="8" t="n">
         <f aca="false">B7*B8</f>
         <v>8000</v>
       </c>
       <c r="D14" s="11" t="n">
         <f aca="false">C14/$C$17</f>
-        <v>0.296296296296296</v>
+        <v>0.34962962962963</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="B15" s="9" t="s">
+      <c r="A15" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="C15" s="10" t="n">
-        <f aca="false">(B6-C14)*B9</f>
-        <v>9500</v>
+      <c r="B15" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="C15" s="8" t="n">
+        <f aca="false">(B11-C14)*B9</f>
+        <v>7440.6779661017</v>
       </c>
       <c r="D15" s="11" t="n">
         <f aca="false">C15/$C$17</f>
-        <v>0.351851851851852</v>
+        <v>0.325185185185185</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="B16" s="9" t="s">
+      <c r="A16" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="C16" s="10" t="n">
-        <f aca="false">B6-C14-C15</f>
-        <v>9500</v>
+      <c r="B16" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="C16" s="8" t="n">
+        <f aca="false">B11-C14-C15</f>
+        <v>7440.6779661017</v>
       </c>
       <c r="D16" s="11" t="n">
         <f aca="false">C16/$C$17</f>
-        <v>0.351851851851852</v>
+        <v>0.325185185185185</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="12" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C17" s="13" t="n">
         <f aca="false">C14+C15+C16</f>
-        <v>27000</v>
+        <v>22881.3559322034</v>
       </c>
       <c r="D17" s="14" t="n">
         <f aca="false">C17/$C$17</f>
@@ -714,33 +726,33 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="12" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C18" s="13" t="n">
         <f aca="false">C17*B10</f>
-        <v>4860</v>
+        <v>4118.64406779661</v>
       </c>
       <c r="D18" s="12"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C19" s="13" t="n">
         <f aca="false">C17+C18</f>
-        <v>31860</v>
+        <v>27000</v>
       </c>
       <c r="D19" s="12"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="0" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C21" s="3" t="str">
         <f aca="false">IF(C16&lt;0,"El monto no alcanza","OK - el detalle suma el monto tope")</f>

</xml_diff>